<commit_message>
Added OrgChartPae]ge.jsx and connected it with App.jsx
</commit_message>
<xml_diff>
--- a/backend/employees.xlsx
+++ b/backend/employees.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/a2fcda027fa75c22/Pictures/Documents/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\GeniusLab-Org-chart\backend\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="83" documentId="8_{8C9FD40E-36F5-4350-9C8C-57B131FACC66}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{17A61B66-6029-4980-8355-CF70086D748E}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8B96CEBE-FDB9-44A3-8D2C-785FF2E32E0C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="10" yWindow="10" windowWidth="19190" windowHeight="11270" xr2:uid="{0A2C4B03-784F-4F64-ABB0-80B2C1608A8D}"/>
   </bookViews>
@@ -211,10 +211,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -580,7 +576,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="2" spans="1:6" ht="29" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A2" s="2">
         <v>100</v>
       </c>
@@ -598,7 +594,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:6" ht="29" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A3" s="2">
         <v>101</v>
       </c>
@@ -618,7 +614,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="4" spans="1:6" ht="29" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
       <c r="A4" s="2">
         <v>102</v>
       </c>

</xml_diff>